<commit_message>
Enhanced ETL framework with logger and updates
</commit_message>
<xml_diff>
--- a/config/test_cases.xlsx
+++ b/config/test_cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\prade\Downloads\etl_framework (1)\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218EFA72-993F-46FA-B9DF-7D5FB0A0C73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B7E776-2A59-4931-8157-21ABB62E9838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>source_type</t>
   </si>
@@ -120,12 +120,24 @@
   <si>
     <t>C:\\Users\\prade\\Downloads\\etl_framework (1)\\target_files\\new_target_data.csv</t>
   </si>
+  <si>
+    <t>primary_key</t>
+  </si>
+  <si>
+    <t>customer_id,account_id,txn_id</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>cust_id,acc_id,txn_id</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,6 +153,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -150,7 +169,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -173,17 +192,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -489,7 +526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -500,9 +537,10 @@
     <col min="6" max="6" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -530,63 +568,72 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="I3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" t="s">
-        <v>10</v>
+      <c r="J3" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>